<commit_message>
Excel temizlendi - yuklenenler kaldirildi
</commit_message>
<xml_diff>
--- a/clenq_trendyol.xlsx
+++ b/clenq_trendyol.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="740" windowWidth="38400" windowHeight="17160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ürünlerinizi Burada Listeleyin" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Urun_Ozellik_Bilgileri" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Menşei Ülke Kısaltmaları" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ürün Denetim Bilgileri" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yardım" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Ürünlerinizi Burada Listeleyin" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Urun_Ozellik_Bilgileri" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Menşei Ülke Kısaltmaları" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Ürün Denetim Bilgileri" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Yardım" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1309,7 +1309,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>4</col>
@@ -1327,24 +1327,24 @@
       <nvPicPr>
         <cNvPr id="3" name="Resim 2"/>
         <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+          <a:picLocks noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:xfrm>
           <a:off x="8900160" y="0"/>
           <a:ext cx="2506980" cy="1880235"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+        <a:prstGeom prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -1974,1630 +1974,14 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001-S</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CLENQ</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>604</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>TRY</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>CLENQ Attack on Titan Oversize Unisex Baskılı Tişört</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;ul&gt;
-&lt;li&gt;Oversize kesimiyle günlük kullanım için rahat ve modern bir görünüm sunan unisex baskılı tişört.&lt;/li&gt;
-&lt;li&gt;Attack on Titan, Shingeki no Kyojin anime ve manga temalı tasarım ile günlük kombinlerinize karakter katar.&lt;/li&gt;
-&lt;li&gt;Yumuşak pamuklu kumaş yapısı sayesinde gün boyu konforlu bir kullanım sağlar.&lt;/li&gt;
-&lt;li&gt;Kısa kollu ve bisiklet yaka tasarımıyla sade, modern ve zamansız bir stile sahiptir.&lt;/li&gt;
-&lt;li&gt;Canlı ve dikkat çekici baskı detayıyla jean, şort, eşofman veya oversize kombinlerle kolayca tamamlanabilir.&lt;/li&gt;
-&lt;li&gt;Unisex kalıbı sayesinde kadın ve erkek kullanıma uygundur.&lt;/li&gt;
-&lt;li&gt;Standart boy uzunluğu ve rahat kalıbı ile farklı vücut tiplerine uyum sağlar.&lt;/li&gt;
-&lt;li&gt;Günlük kullanım, konser, festival, sokak stili ve casual kombinler için ideal bir parçadır.&lt;/li&gt;
-&lt;li&gt;Baskının uzun ömürlü olması için ürünün ters çevrilerek 30 derecede yıkanması önerilir.&lt;/li&gt;
-&lt;li&gt;Ürün baskılı olduğu için doğrudan baskı üzerine ütü yapılmamalıdır.&lt;/li&gt;
-&lt;li&gt;Paket içeriği 1 adet baskılı tişörtten oluşmaktadır.&lt;/li&gt;
-&lt;li&gt;Türkiye'de üretilmiştir.&lt;/li&gt;
-&lt;/ul&gt;&lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>850</v>
-      </c>
-      <c r="I2" t="n">
-        <v>850</v>
-      </c>
-      <c r="J2" t="n">
-        <v>99</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001-S</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
-        <v>20</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-model_on.jpg</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-aski-on.jpg</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-beden.jpg</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-iscilik.jpg</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-kalip.jpg</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-pamuk.jpg</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>DTF Baskı</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>Kısa Kol</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>Baskılı</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>Standart</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>Süprem</t>
-        </is>
-      </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>Cepsiz</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>Dokuma</t>
-        </is>
-      </c>
-      <c r="AZ2" t="inlineStr">
-        <is>
-          <t>%100 Pamuk</t>
-        </is>
-      </c>
-      <c r="BA2" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="BB2" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="BC2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG2" t="inlineStr">
-        <is>
-          <t>Tüm Sezonlar</t>
-        </is>
-      </c>
-      <c r="BH2" t="inlineStr">
-        <is>
-          <t>Ek Özellik Mevcut Değil</t>
-        </is>
-      </c>
-      <c r="BL2" t="inlineStr">
-        <is>
-          <t>Kutu yok</t>
-        </is>
-      </c>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>Bisiklet Yaka</t>
-        </is>
-      </c>
-      <c r="BP2" t="inlineStr">
-        <is>
-          <t>Unisex</t>
-        </is>
-      </c>
-      <c r="BQ2" t="inlineStr">
-        <is>
-          <t>Yetişkin</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001-M</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CLENQ</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>604</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>TRY</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CLENQ Attack on Titan Oversize Unisex Baskılı Tişört</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;ul&gt;
-&lt;li&gt;Oversize kesimiyle günlük kullanım için rahat ve modern bir görünüm sunan unisex baskılı tişört.&lt;/li&gt;
-&lt;li&gt;Attack on Titan, Shingeki no Kyojin anime ve manga temalı tasarım ile günlük kombinlerinize karakter katar.&lt;/li&gt;
-&lt;li&gt;Yumuşak pamuklu kumaş yapısı sayesinde gün boyu konforlu bir kullanım sağlar.&lt;/li&gt;
-&lt;li&gt;Kısa kollu ve bisiklet yaka tasarımıyla sade, modern ve zamansız bir stile sahiptir.&lt;/li&gt;
-&lt;li&gt;Canlı ve dikkat çekici baskı detayıyla jean, şort, eşofman veya oversize kombinlerle kolayca tamamlanabilir.&lt;/li&gt;
-&lt;li&gt;Unisex kalıbı sayesinde kadın ve erkek kullanıma uygundur.&lt;/li&gt;
-&lt;li&gt;Standart boy uzunluğu ve rahat kalıbı ile farklı vücut tiplerine uyum sağlar.&lt;/li&gt;
-&lt;li&gt;Günlük kullanım, konser, festival, sokak stili ve casual kombinler için ideal bir parçadır.&lt;/li&gt;
-&lt;li&gt;Baskının uzun ömürlü olması için ürünün ters çevrilerek 30 derecede yıkanması önerilir.&lt;/li&gt;
-&lt;li&gt;Ürün baskılı olduğu için doğrudan baskı üzerine ütü yapılmamalıdır.&lt;/li&gt;
-&lt;li&gt;Paket içeriği 1 adet baskılı tişörtten oluşmaktadır.&lt;/li&gt;
-&lt;li&gt;Türkiye'de üretilmiştir.&lt;/li&gt;
-&lt;/ul&gt;&lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>850</v>
-      </c>
-      <c r="I3" t="n">
-        <v>850</v>
-      </c>
-      <c r="J3" t="n">
-        <v>99</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001-M</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>20</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-model_on.jpg</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-aski-on.jpg</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-beden.jpg</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-iscilik.jpg</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-kalip.jpg</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-pamuk.jpg</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>DTF Baskı</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>Kısa Kol</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>Baskılı</t>
-        </is>
-      </c>
-      <c r="AJ3" t="inlineStr">
-        <is>
-          <t>Standart</t>
-        </is>
-      </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>Süprem</t>
-        </is>
-      </c>
-      <c r="AP3" t="inlineStr">
-        <is>
-          <t>Cepsiz</t>
-        </is>
-      </c>
-      <c r="AQ3" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="AS3" t="inlineStr">
-        <is>
-          <t>Dokuma</t>
-        </is>
-      </c>
-      <c r="AZ3" t="inlineStr">
-        <is>
-          <t>%100 Pamuk</t>
-        </is>
-      </c>
-      <c r="BA3" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="BB3" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="BC3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG3" t="inlineStr">
-        <is>
-          <t>Tüm Sezonlar</t>
-        </is>
-      </c>
-      <c r="BH3" t="inlineStr">
-        <is>
-          <t>Ek Özellik Mevcut Değil</t>
-        </is>
-      </c>
-      <c r="BL3" t="inlineStr">
-        <is>
-          <t>Kutu yok</t>
-        </is>
-      </c>
-      <c r="BN3" t="inlineStr">
-        <is>
-          <t>Bisiklet Yaka</t>
-        </is>
-      </c>
-      <c r="BP3" t="inlineStr">
-        <is>
-          <t>Unisex</t>
-        </is>
-      </c>
-      <c r="BQ3" t="inlineStr">
-        <is>
-          <t>Yetişkin</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001-L</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CLENQ</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>604</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>TRY</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>CLENQ Attack on Titan Oversize Unisex Baskılı Tişört</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;ul&gt;
-&lt;li&gt;Oversize kesimiyle günlük kullanım için rahat ve modern bir görünüm sunan unisex baskılı tişört.&lt;/li&gt;
-&lt;li&gt;Attack on Titan, Shingeki no Kyojin anime ve manga temalı tasarım ile günlük kombinlerinize karakter katar.&lt;/li&gt;
-&lt;li&gt;Yumuşak pamuklu kumaş yapısı sayesinde gün boyu konforlu bir kullanım sağlar.&lt;/li&gt;
-&lt;li&gt;Kısa kollu ve bisiklet yaka tasarımıyla sade, modern ve zamansız bir stile sahiptir.&lt;/li&gt;
-&lt;li&gt;Canlı ve dikkat çekici baskı detayıyla jean, şort, eşofman veya oversize kombinlerle kolayca tamamlanabilir.&lt;/li&gt;
-&lt;li&gt;Unisex kalıbı sayesinde kadın ve erkek kullanıma uygundur.&lt;/li&gt;
-&lt;li&gt;Standart boy uzunluğu ve rahat kalıbı ile farklı vücut tiplerine uyum sağlar.&lt;/li&gt;
-&lt;li&gt;Günlük kullanım, konser, festival, sokak stili ve casual kombinler için ideal bir parçadır.&lt;/li&gt;
-&lt;li&gt;Baskının uzun ömürlü olması için ürünün ters çevrilerek 30 derecede yıkanması önerilir.&lt;/li&gt;
-&lt;li&gt;Ürün baskılı olduğu için doğrudan baskı üzerine ütü yapılmamalıdır.&lt;/li&gt;
-&lt;li&gt;Paket içeriği 1 adet baskılı tişörtten oluşmaktadır.&lt;/li&gt;
-&lt;li&gt;Türkiye'de üretilmiştir.&lt;/li&gt;
-&lt;/ul&gt;&lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>850</v>
-      </c>
-      <c r="I4" t="n">
-        <v>850</v>
-      </c>
-      <c r="J4" t="n">
-        <v>99</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001-L</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>20</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-model_on.jpg</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-aski-on.jpg</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-beden.jpg</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-iscilik.jpg</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-kalip.jpg</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-pamuk.jpg</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>DTF Baskı</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>Kısa Kol</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>Baskılı</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>Standart</t>
-        </is>
-      </c>
-      <c r="AM4" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AN4" t="inlineStr">
-        <is>
-          <t>Süprem</t>
-        </is>
-      </c>
-      <c r="AP4" t="inlineStr">
-        <is>
-          <t>Cepsiz</t>
-        </is>
-      </c>
-      <c r="AQ4" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="AS4" t="inlineStr">
-        <is>
-          <t>Dokuma</t>
-        </is>
-      </c>
-      <c r="AZ4" t="inlineStr">
-        <is>
-          <t>%100 Pamuk</t>
-        </is>
-      </c>
-      <c r="BA4" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="BB4" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="BC4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG4" t="inlineStr">
-        <is>
-          <t>Tüm Sezonlar</t>
-        </is>
-      </c>
-      <c r="BH4" t="inlineStr">
-        <is>
-          <t>Ek Özellik Mevcut Değil</t>
-        </is>
-      </c>
-      <c r="BL4" t="inlineStr">
-        <is>
-          <t>Kutu yok</t>
-        </is>
-      </c>
-      <c r="BN4" t="inlineStr">
-        <is>
-          <t>Bisiklet Yaka</t>
-        </is>
-      </c>
-      <c r="BP4" t="inlineStr">
-        <is>
-          <t>Unisex</t>
-        </is>
-      </c>
-      <c r="BQ4" t="inlineStr">
-        <is>
-          <t>Yetişkin</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001-XL</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CLENQ</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>604</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>TRY</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>CLENQ Attack on Titan Oversize Unisex Baskılı Tişört</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;ul&gt;
-&lt;li&gt;Oversize kesimiyle günlük kullanım için rahat ve modern bir görünüm sunan unisex baskılı tişört.&lt;/li&gt;
-&lt;li&gt;Attack on Titan, Shingeki no Kyojin anime ve manga temalı tasarım ile günlük kombinlerinize karakter katar.&lt;/li&gt;
-&lt;li&gt;Yumuşak pamuklu kumaş yapısı sayesinde gün boyu konforlu bir kullanım sağlar.&lt;/li&gt;
-&lt;li&gt;Kısa kollu ve bisiklet yaka tasarımıyla sade, modern ve zamansız bir stile sahiptir.&lt;/li&gt;
-&lt;li&gt;Canlı ve dikkat çekici baskı detayıyla jean, şort, eşofman veya oversize kombinlerle kolayca tamamlanabilir.&lt;/li&gt;
-&lt;li&gt;Unisex kalıbı sayesinde kadın ve erkek kullanıma uygundur.&lt;/li&gt;
-&lt;li&gt;Standart boy uzunluğu ve rahat kalıbı ile farklı vücut tiplerine uyum sağlar.&lt;/li&gt;
-&lt;li&gt;Günlük kullanım, konser, festival, sokak stili ve casual kombinler için ideal bir parçadır.&lt;/li&gt;
-&lt;li&gt;Baskının uzun ömürlü olması için ürünün ters çevrilerek 30 derecede yıkanması önerilir.&lt;/li&gt;
-&lt;li&gt;Ürün baskılı olduğu için doğrudan baskı üzerine ütü yapılmamalıdır.&lt;/li&gt;
-&lt;li&gt;Paket içeriği 1 adet baskılı tişörtten oluşmaktadır.&lt;/li&gt;
-&lt;li&gt;Türkiye'de üretilmiştir.&lt;/li&gt;
-&lt;/ul&gt;&lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>850</v>
-      </c>
-      <c r="I5" t="n">
-        <v>850</v>
-      </c>
-      <c r="J5" t="n">
-        <v>99</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>CLENQ-AOT-TITAN-001-XL</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>20</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-model_on.jpg</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-aski-on.jpg</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-beden.jpg</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-iscilik.jpg</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-kalip.jpg</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-AOT-TITAN-001/CLENQ-AOT-TITAN-001-pamuk.jpg</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>DTF Baskı</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>Kısa Kol</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>Baskılı</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>Standart</t>
-        </is>
-      </c>
-      <c r="AM5" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AN5" t="inlineStr">
-        <is>
-          <t>Süprem</t>
-        </is>
-      </c>
-      <c r="AP5" t="inlineStr">
-        <is>
-          <t>Cepsiz</t>
-        </is>
-      </c>
-      <c r="AQ5" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="AS5" t="inlineStr">
-        <is>
-          <t>Dokuma</t>
-        </is>
-      </c>
-      <c r="AZ5" t="inlineStr">
-        <is>
-          <t>%100 Pamuk</t>
-        </is>
-      </c>
-      <c r="BA5" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="BB5" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="BC5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG5" t="inlineStr">
-        <is>
-          <t>Tüm Sezonlar</t>
-        </is>
-      </c>
-      <c r="BH5" t="inlineStr">
-        <is>
-          <t>Ek Özellik Mevcut Değil</t>
-        </is>
-      </c>
-      <c r="BL5" t="inlineStr">
-        <is>
-          <t>Kutu yok</t>
-        </is>
-      </c>
-      <c r="BN5" t="inlineStr">
-        <is>
-          <t>Bisiklet Yaka</t>
-        </is>
-      </c>
-      <c r="BP5" t="inlineStr">
-        <is>
-          <t>Unisex</t>
-        </is>
-      </c>
-      <c r="BQ5" t="inlineStr">
-        <is>
-          <t>Yetişkin</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001-S</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CLENQ</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>604</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>TRY</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>CLENQ Wolf Emblem Oversize Unisex Baskılı Tişört</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;ul&gt;
-&lt;li&gt;Oversize kesimiyle günlük kullanım için rahat ve modern bir görünüm sunan unisex baskılı tişört.&lt;/li&gt;
-&lt;li&gt;Kurt ve tribal temalı, mistik amblem tasarımıyla günlük kombinlerinize güçlü bir karakter katar.&lt;/li&gt;
-&lt;li&gt;Yumuşak pamuklu kumaş yapısı sayesinde gün boyu konforlu bir kullanım sağlar.&lt;/li&gt;
-&lt;li&gt;Kısa kollu ve bisiklet yaka tasarımıyla sade, modern ve zamansız bir stile sahiptir.&lt;/li&gt;
-&lt;li&gt;Canlı ve dikkat çekici baskı detayıyla jean, şort, eşofman veya oversize kombinlerle kolayca tamamlanabilir.&lt;/li&gt;
-&lt;li&gt;Unisex kalıbı sayesinde kadın ve erkek kullanıma uygundur.&lt;/li&gt;
-&lt;li&gt;Standart boy uzunluğu ve rahat kalıbı ile farklı vücut tiplerine uyum sağlar.&lt;/li&gt;
-&lt;li&gt;Günlük kullanım, konser, festival, sokak stili ve casual kombinler için ideal bir parçadır.&lt;/li&gt;
-&lt;li&gt;Baskının uzun ömürlü olması için ürünün ters çevrilerek 30 derecede yıkanması önerilir.&lt;/li&gt;
-&lt;li&gt;Ürün baskılı olduğu için doğrudan baskı üzerine ütü yapılmamalıdır.&lt;/li&gt;
-&lt;li&gt;Paket içeriği 1 adet baskılı tişörtten oluşmaktadır.&lt;/li&gt;
-&lt;li&gt;Türkiye'de üretilmiştir.&lt;/li&gt;
-&lt;/ul&gt;&lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>850</v>
-      </c>
-      <c r="I6" t="n">
-        <v>850</v>
-      </c>
-      <c r="J6" t="n">
-        <v>99</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001-S</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>20</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-model_on.jpg</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-aski-on.jpg</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-beden.jpg</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-iscilik.jpg</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-kalip.jpg</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-pamuk.jpg</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>DTF Baskı</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>Kısa Kol</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>Baskılı</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr">
-        <is>
-          <t>Standart</t>
-        </is>
-      </c>
-      <c r="AM6" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AN6" t="inlineStr">
-        <is>
-          <t>Süprem</t>
-        </is>
-      </c>
-      <c r="AP6" t="inlineStr">
-        <is>
-          <t>Cepsiz</t>
-        </is>
-      </c>
-      <c r="AQ6" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="AS6" t="inlineStr">
-        <is>
-          <t>Dokuma</t>
-        </is>
-      </c>
-      <c r="AZ6" t="inlineStr">
-        <is>
-          <t>%100 Pamuk</t>
-        </is>
-      </c>
-      <c r="BA6" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="BB6" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="BC6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG6" t="inlineStr">
-        <is>
-          <t>Tüm Sezonlar</t>
-        </is>
-      </c>
-      <c r="BH6" t="inlineStr">
-        <is>
-          <t>Ek Özellik Mevcut Değil</t>
-        </is>
-      </c>
-      <c r="BL6" t="inlineStr">
-        <is>
-          <t>Kutu yok</t>
-        </is>
-      </c>
-      <c r="BN6" t="inlineStr">
-        <is>
-          <t>Bisiklet Yaka</t>
-        </is>
-      </c>
-      <c r="BP6" t="inlineStr">
-        <is>
-          <t>Unisex</t>
-        </is>
-      </c>
-      <c r="BQ6" t="inlineStr">
-        <is>
-          <t>Yetişkin</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001-M</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CLENQ</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>604</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>TRY</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>CLENQ Wolf Emblem Oversize Unisex Baskılı Tişört</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;ul&gt;
-&lt;li&gt;Oversize kesimiyle günlük kullanım için rahat ve modern bir görünüm sunan unisex baskılı tişört.&lt;/li&gt;
-&lt;li&gt;Kurt ve tribal temalı, mistik amblem tasarımıyla günlük kombinlerinize güçlü bir karakter katar.&lt;/li&gt;
-&lt;li&gt;Yumuşak pamuklu kumaş yapısı sayesinde gün boyu konforlu bir kullanım sağlar.&lt;/li&gt;
-&lt;li&gt;Kısa kollu ve bisiklet yaka tasarımıyla sade, modern ve zamansız bir stile sahiptir.&lt;/li&gt;
-&lt;li&gt;Canlı ve dikkat çekici baskı detayıyla jean, şort, eşofman veya oversize kombinlerle kolayca tamamlanabilir.&lt;/li&gt;
-&lt;li&gt;Unisex kalıbı sayesinde kadın ve erkek kullanıma uygundur.&lt;/li&gt;
-&lt;li&gt;Standart boy uzunluğu ve rahat kalıbı ile farklı vücut tiplerine uyum sağlar.&lt;/li&gt;
-&lt;li&gt;Günlük kullanım, konser, festival, sokak stili ve casual kombinler için ideal bir parçadır.&lt;/li&gt;
-&lt;li&gt;Baskının uzun ömürlü olması için ürünün ters çevrilerek 30 derecede yıkanması önerilir.&lt;/li&gt;
-&lt;li&gt;Ürün baskılı olduğu için doğrudan baskı üzerine ütü yapılmamalıdır.&lt;/li&gt;
-&lt;li&gt;Paket içeriği 1 adet baskılı tişörtten oluşmaktadır.&lt;/li&gt;
-&lt;li&gt;Türkiye'de üretilmiştir.&lt;/li&gt;
-&lt;/ul&gt;&lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>850</v>
-      </c>
-      <c r="I7" t="n">
-        <v>850</v>
-      </c>
-      <c r="J7" t="n">
-        <v>99</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001-M</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>20</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-model_on.jpg</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-aski-on.jpg</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-beden.jpg</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-iscilik.jpg</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-kalip.jpg</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-pamuk.jpg</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>DTF Baskı</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>Kısa Kol</t>
-        </is>
-      </c>
-      <c r="AI7" t="inlineStr">
-        <is>
-          <t>Baskılı</t>
-        </is>
-      </c>
-      <c r="AJ7" t="inlineStr">
-        <is>
-          <t>Standart</t>
-        </is>
-      </c>
-      <c r="AM7" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AN7" t="inlineStr">
-        <is>
-          <t>Süprem</t>
-        </is>
-      </c>
-      <c r="AP7" t="inlineStr">
-        <is>
-          <t>Cepsiz</t>
-        </is>
-      </c>
-      <c r="AQ7" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="AS7" t="inlineStr">
-        <is>
-          <t>Dokuma</t>
-        </is>
-      </c>
-      <c r="AZ7" t="inlineStr">
-        <is>
-          <t>%100 Pamuk</t>
-        </is>
-      </c>
-      <c r="BA7" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="BB7" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="BC7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG7" t="inlineStr">
-        <is>
-          <t>Tüm Sezonlar</t>
-        </is>
-      </c>
-      <c r="BH7" t="inlineStr">
-        <is>
-          <t>Ek Özellik Mevcut Değil</t>
-        </is>
-      </c>
-      <c r="BL7" t="inlineStr">
-        <is>
-          <t>Kutu yok</t>
-        </is>
-      </c>
-      <c r="BN7" t="inlineStr">
-        <is>
-          <t>Bisiklet Yaka</t>
-        </is>
-      </c>
-      <c r="BP7" t="inlineStr">
-        <is>
-          <t>Unisex</t>
-        </is>
-      </c>
-      <c r="BQ7" t="inlineStr">
-        <is>
-          <t>Yetişkin</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001-L</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CLENQ</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>604</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>TRY</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>CLENQ Wolf Emblem Oversize Unisex Baskılı Tişört</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;ul&gt;
-&lt;li&gt;Oversize kesimiyle günlük kullanım için rahat ve modern bir görünüm sunan unisex baskılı tişört.&lt;/li&gt;
-&lt;li&gt;Kurt ve tribal temalı, mistik amblem tasarımıyla günlük kombinlerinize güçlü bir karakter katar.&lt;/li&gt;
-&lt;li&gt;Yumuşak pamuklu kumaş yapısı sayesinde gün boyu konforlu bir kullanım sağlar.&lt;/li&gt;
-&lt;li&gt;Kısa kollu ve bisiklet yaka tasarımıyla sade, modern ve zamansız bir stile sahiptir.&lt;/li&gt;
-&lt;li&gt;Canlı ve dikkat çekici baskı detayıyla jean, şort, eşofman veya oversize kombinlerle kolayca tamamlanabilir.&lt;/li&gt;
-&lt;li&gt;Unisex kalıbı sayesinde kadın ve erkek kullanıma uygundur.&lt;/li&gt;
-&lt;li&gt;Standart boy uzunluğu ve rahat kalıbı ile farklı vücut tiplerine uyum sağlar.&lt;/li&gt;
-&lt;li&gt;Günlük kullanım, konser, festival, sokak stili ve casual kombinler için ideal bir parçadır.&lt;/li&gt;
-&lt;li&gt;Baskının uzun ömürlü olması için ürünün ters çevrilerek 30 derecede yıkanması önerilir.&lt;/li&gt;
-&lt;li&gt;Ürün baskılı olduğu için doğrudan baskı üzerine ütü yapılmamalıdır.&lt;/li&gt;
-&lt;li&gt;Paket içeriği 1 adet baskılı tişörtten oluşmaktadır.&lt;/li&gt;
-&lt;li&gt;Türkiye'de üretilmiştir.&lt;/li&gt;
-&lt;/ul&gt;&lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>850</v>
-      </c>
-      <c r="I8" t="n">
-        <v>850</v>
-      </c>
-      <c r="J8" t="n">
-        <v>99</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001-L</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>20</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-model_on.jpg</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-aski-on.jpg</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-beden.jpg</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-iscilik.jpg</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-kalip.jpg</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-pamuk.jpg</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>DTF Baskı</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>Kısa Kol</t>
-        </is>
-      </c>
-      <c r="AI8" t="inlineStr">
-        <is>
-          <t>Baskılı</t>
-        </is>
-      </c>
-      <c r="AJ8" t="inlineStr">
-        <is>
-          <t>Standart</t>
-        </is>
-      </c>
-      <c r="AM8" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AN8" t="inlineStr">
-        <is>
-          <t>Süprem</t>
-        </is>
-      </c>
-      <c r="AP8" t="inlineStr">
-        <is>
-          <t>Cepsiz</t>
-        </is>
-      </c>
-      <c r="AQ8" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="AS8" t="inlineStr">
-        <is>
-          <t>Dokuma</t>
-        </is>
-      </c>
-      <c r="AZ8" t="inlineStr">
-        <is>
-          <t>%100 Pamuk</t>
-        </is>
-      </c>
-      <c r="BA8" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="BB8" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="BC8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG8" t="inlineStr">
-        <is>
-          <t>Tüm Sezonlar</t>
-        </is>
-      </c>
-      <c r="BH8" t="inlineStr">
-        <is>
-          <t>Ek Özellik Mevcut Değil</t>
-        </is>
-      </c>
-      <c r="BL8" t="inlineStr">
-        <is>
-          <t>Kutu yok</t>
-        </is>
-      </c>
-      <c r="BN8" t="inlineStr">
-        <is>
-          <t>Bisiklet Yaka</t>
-        </is>
-      </c>
-      <c r="BP8" t="inlineStr">
-        <is>
-          <t>Unisex</t>
-        </is>
-      </c>
-      <c r="BQ8" t="inlineStr">
-        <is>
-          <t>Yetişkin</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001-XL</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CLENQ</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>604</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>TRY</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>CLENQ Wolf Emblem Oversize Unisex Baskılı Tişört</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;ul&gt;
-&lt;li&gt;Oversize kesimiyle günlük kullanım için rahat ve modern bir görünüm sunan unisex baskılı tişört.&lt;/li&gt;
-&lt;li&gt;Kurt ve tribal temalı, mistik amblem tasarımıyla günlük kombinlerinize güçlü bir karakter katar.&lt;/li&gt;
-&lt;li&gt;Yumuşak pamuklu kumaş yapısı sayesinde gün boyu konforlu bir kullanım sağlar.&lt;/li&gt;
-&lt;li&gt;Kısa kollu ve bisiklet yaka tasarımıyla sade, modern ve zamansız bir stile sahiptir.&lt;/li&gt;
-&lt;li&gt;Canlı ve dikkat çekici baskı detayıyla jean, şort, eşofman veya oversize kombinlerle kolayca tamamlanabilir.&lt;/li&gt;
-&lt;li&gt;Unisex kalıbı sayesinde kadın ve erkek kullanıma uygundur.&lt;/li&gt;
-&lt;li&gt;Standart boy uzunluğu ve rahat kalıbı ile farklı vücut tiplerine uyum sağlar.&lt;/li&gt;
-&lt;li&gt;Günlük kullanım, konser, festival, sokak stili ve casual kombinler için ideal bir parçadır.&lt;/li&gt;
-&lt;li&gt;Baskının uzun ömürlü olması için ürünün ters çevrilerek 30 derecede yıkanması önerilir.&lt;/li&gt;
-&lt;li&gt;Ürün baskılı olduğu için doğrudan baskı üzerine ütü yapılmamalıdır.&lt;/li&gt;
-&lt;li&gt;Paket içeriği 1 adet baskılı tişörtten oluşmaktadır.&lt;/li&gt;
-&lt;li&gt;Türkiye'de üretilmiştir.&lt;/li&gt;
-&lt;/ul&gt;&lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>850</v>
-      </c>
-      <c r="I9" t="n">
-        <v>850</v>
-      </c>
-      <c r="J9" t="n">
-        <v>99</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>CLENQ-WOLF-EMBLEM-001-XL</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>20</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-model_on.jpg</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-aski-on.jpg</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-beden.jpg</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-iscilik.jpg</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-kalip.jpg</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/dmrern/clenq-gorseller/main/CLENQ-WOLF-EMBLEM-001/CLENQ-WOLF-EMBLEM-001-pamuk.jpg</t>
-        </is>
-      </c>
-      <c r="Z9" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>DTF Baskı</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>Kısa Kol</t>
-        </is>
-      </c>
-      <c r="AI9" t="inlineStr">
-        <is>
-          <t>Baskılı</t>
-        </is>
-      </c>
-      <c r="AJ9" t="inlineStr">
-        <is>
-          <t>Standart</t>
-        </is>
-      </c>
-      <c r="AM9" t="inlineStr">
-        <is>
-          <t>Oversize</t>
-        </is>
-      </c>
-      <c r="AN9" t="inlineStr">
-        <is>
-          <t>Süprem</t>
-        </is>
-      </c>
-      <c r="AP9" t="inlineStr">
-        <is>
-          <t>Cepsiz</t>
-        </is>
-      </c>
-      <c r="AQ9" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="AS9" t="inlineStr">
-        <is>
-          <t>Dokuma</t>
-        </is>
-      </c>
-      <c r="AZ9" t="inlineStr">
-        <is>
-          <t>%100 Pamuk</t>
-        </is>
-      </c>
-      <c r="BA9" t="inlineStr">
-        <is>
-          <t>Siyah</t>
-        </is>
-      </c>
-      <c r="BB9" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="BC9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG9" t="inlineStr">
-        <is>
-          <t>Tüm Sezonlar</t>
-        </is>
-      </c>
-      <c r="BH9" t="inlineStr">
-        <is>
-          <t>Ek Özellik Mevcut Değil</t>
-        </is>
-      </c>
-      <c r="BL9" t="inlineStr">
-        <is>
-          <t>Kutu yok</t>
-        </is>
-      </c>
-      <c r="BN9" t="inlineStr">
-        <is>
-          <t>Bisiklet Yaka</t>
-        </is>
-      </c>
-      <c r="BP9" t="inlineStr">
-        <is>
-          <t>Unisex</t>
-        </is>
-      </c>
-      <c r="BQ9" t="inlineStr">
-        <is>
-          <t>Yetişkin</t>
-        </is>
-      </c>
-    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
   </sheetData>
   <dataValidations count="51">
     <dataValidation sqref="AC2:AC1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="DEĞER SEÇİMİ HATASI" error="Sadece izin verilen değerleri girebilirsiniz. Lütfen kontrol ediniz." type="list" errorStyle="stop">

</xml_diff>